<commit_message>
feat: scraping por batches de 20 chats con fetchMessageHistory
</commit_message>
<xml_diff>
--- a/lipo_blue_2026-07-18.xlsx
+++ b/lipo_blue_2026-07-18.xlsx
@@ -397,59 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="25.83203125" customWidth="1"/>
     <col min="4" max="4" width="30.83203125" customWidth="1"/>
-    <col min="5" max="5" width="50.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="60.83203125" customWidth="1"/>
+    <col min="6" max="6" width="25.83203125" customWidth="1"/>
   </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Chat</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Es Grupo</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Contacto/Nombre</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Numero/JID</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Mensaje</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Fecha</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>status@broadcast</v>
-      </c>
-      <c r="B2" t="str">
-        <v>No</v>
-      </c>
-      <c r="C2" t="str">
-        <v/>
-      </c>
-      <c r="D2" t="str">
-        <v>6227719368922@lid</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Un atardecer 🌹🙏con mi ♥️</v>
-      </c>
-      <c r="F2" t="str">
-        <v>18/7/2026, 3:51:15 p. m.</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>